<commit_message>
Release 2.2.0: compact fleet UI, bulk control and Android parity
</commit_message>
<xml_diff>
--- a/docs/testing/asic_acceptance.xlsx
+++ b/docs/testing/asic_acceptance.xlsx
@@ -1509,7 +1509,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Укажите модель</t>
+          <t>Antminer S21_i (web: S21)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1519,12 +1519,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Заполнить</t>
+          <t>PitBit.78 / incm.C074; Fri Feb 2 17:03:40 CST 2024</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Заполнить</t>
+          <t>AMLCtrl_BHB68XXX / API 3.1 / ASIC Monitor 2.1.0 source 2026-10-03</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1544,12 +1544,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Не проверено</t>
+          <t>✓ Пройден</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Не проверено</t>
+          <t>✓ Пройден</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1601,7 +1601,11 @@
         <f>COUNTIF(E13:R13,"✓ Пройден")</f>
         <v/>
       </c>
-      <c r="T13" s="3" t="str"/>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>03.10.2026: docs/testing/pitbit-s21-2026-10-03.md. LED ON/OFF подтверждены API, визуальный осмотр ожидается. Sleep: mode 1, текущий хешрейт 0, stopped. Wakeup: mode 0, майнинг возобновился; номинальный разгон не проверен. Reboot: uptime 142→30 s, прежняя идентичность, появился хешрейт. Полная конфигурация и LED восстановлены. Low/High/HEM не отправлялись. T01 и T06 не отмечены полностью пройденными: полная сверка и штатный разгон не выполнены.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="3" t="inlineStr">

</xml_diff>